<commit_message>
add break_schedule logic with auto break generation
</commit_message>
<xml_diff>
--- a/split_30minute_result.xlsx
+++ b/split_30minute_result.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="シフト" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="欠員ログ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="休憩予定" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -884,7 +885,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Cさん</t>
+          <t>Dさん</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -901,7 +902,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -913,17 +914,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>12:00-12:30</t>
+          <t>12:30-13:00</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Eさん</t>
+          <t>Cさん</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>フロア</t>
+          <t>バリスタ</t>
         </is>
       </c>
     </row>
@@ -935,12 +936,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Cさん</t>
+          <t>Dさん</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>バリスタ</t>
+          <t>キャッシャー</t>
         </is>
       </c>
     </row>
@@ -952,29 +953,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
+          <t>フロア</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>12:30-13:00</t>
+          <t>13:00-13:30</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Eさん</t>
+          <t>Cさん</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>フロア</t>
+          <t>バリスタ</t>
         </is>
       </c>
     </row>
@@ -986,46 +987,46 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Dさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>バリスタ</t>
+          <t>キャッシャー</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>13:00-13:30</t>
+          <t>13:30-14:00</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cさん</t>
+          <t>Dさん</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
+          <t>バリスタ</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>13:00-13:30</t>
+          <t>13:30-14:00</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Eさん</t>
+          <t>Cさん</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>フロア</t>
+          <t>キャッシャー</t>
         </is>
       </c>
     </row>
@@ -1037,46 +1038,46 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Cさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>バリスタ</t>
+          <t>フロア</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>13:30-14:00</t>
+          <t>14:00-14:30</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Dさん</t>
+          <t>Cさん</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
+          <t>バリスタ</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>13:30-14:00</t>
+          <t>14:00-14:30</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Eさん</t>
+          <t>Dさん</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>フロア</t>
+          <t>キャッシャー</t>
         </is>
       </c>
     </row>
@@ -1088,19 +1089,19 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>バリスタ</t>
+          <t>フロア</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>14:00-14:30</t>
+          <t>14:30-15:00</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1110,7 +1111,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
+          <t>バリスタ</t>
         </is>
       </c>
     </row>
@@ -1122,41 +1123,41 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Dさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>バリスタ</t>
+          <t>キャッシャー</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>14:30-15:00</t>
+          <t>15:00-15:30</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Eさん</t>
+          <t>Fさん</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
+          <t>バリスタ</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>15:00-15:30</t>
+          <t>15:30-16:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Eさん</t>
+          <t>Fさん</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1168,131 +1169,131 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>15:00-15:30</t>
+          <t>16:00-16:30</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Fさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
+          <t>バリスタ</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>15:30-16:00</t>
+          <t>16:00-16:30</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Eさん</t>
+          <t>Fさん</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>バリスタ</t>
+          <t>キャッシャー</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>15:30-16:00</t>
+          <t>16:30-17:00</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Fさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
+          <t>バリスタ</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>16:00-16:30</t>
+          <t>16:30-17:00</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Eさん</t>
+          <t>Fさん</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>バリスタ</t>
+          <t>キャッシャー</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>16:00-16:30</t>
+          <t>17:00-17:30</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Fさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
+          <t>バリスタ</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>16:30-17:00</t>
+          <t>17:00-17:30</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Eさん</t>
+          <t>Fさん</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>バリスタ</t>
+          <t>キャッシャー</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>16:30-17:00</t>
+          <t>17:00-17:30</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Fさん</t>
+          <t>Gさん</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
+          <t>フロア</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>17:00-17:30</t>
+          <t>17:30-18:00</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Fさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1304,12 +1305,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>17:00-17:30</t>
+          <t>17:30-18:00</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Eさん</t>
+          <t>Fさん</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1321,7 +1322,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>17:00-17:30</t>
+          <t>17:30-18:00</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1338,12 +1339,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>17:30-18:00</t>
+          <t>18:00-18:30</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Eさん</t>
+          <t>Gさん</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1355,12 +1356,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>17:30-18:00</t>
+          <t>18:00-18:30</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Fさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1372,63 +1373,63 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>17:30-18:00</t>
+          <t>18:30-19:00</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Gさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>フロア</t>
+          <t>バリスタ</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>18:00-18:30</t>
+          <t>18:30-19:00</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Fさん</t>
+          <t>Gさん</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>バリスタ</t>
+          <t>キャッシャー</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>18:00-18:30</t>
+          <t>18:30-19:00</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Gさん</t>
+          <t>Fさん</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
+          <t>フロア</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>18:30-19:00</t>
+          <t>19:00-19:30</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Fさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1440,12 +1441,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>18:30-19:00</t>
+          <t>19:00-19:30</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Gさん</t>
+          <t>Fさん</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1462,46 +1463,46 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Eさん</t>
+          <t>Gさん</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>バリスタ</t>
+          <t>フロア</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>19:00-19:30</t>
+          <t>19:30-20:00</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Fさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
+          <t>バリスタ</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>19:00-19:30</t>
+          <t>19:30-20:00</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Gさん</t>
+          <t>Fさん</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>フロア</t>
+          <t>キャッシャー</t>
         </is>
       </c>
     </row>
@@ -1513,46 +1514,46 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Eさん</t>
+          <t>Gさん</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>バリスタ</t>
+          <t>フロア</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>19:30-20:00</t>
+          <t>20:00-20:30</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Fさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
+          <t>バリスタ</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>19:30-20:00</t>
+          <t>20:00-20:30</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Gさん</t>
+          <t>Fさん</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>フロア</t>
+          <t>キャッシャー</t>
         </is>
       </c>
     </row>
@@ -1564,19 +1565,19 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Eさん</t>
+          <t>Gさん</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>バリスタ</t>
+          <t>フロア</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>20:00-20:30</t>
+          <t>20:30-21:00</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1586,24 +1587,24 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
+          <t>バリスタ</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>20:00-20:30</t>
+          <t>20:30-21:00</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Gさん</t>
+          <t>Eさん</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>フロア</t>
+          <t>キャッシャー</t>
         </is>
       </c>
     </row>
@@ -1615,19 +1616,19 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Fさん</t>
+          <t>Gさん</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>バリスタ</t>
+          <t>フロア</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>20:30-21:00</t>
+          <t>21:00-21:30</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1637,31 +1638,31 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
+          <t>バリスタ</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>20:30-21:00</t>
+          <t>21:00-21:30</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Gさん</t>
+          <t>Fさん</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>フロア</t>
+          <t>キャッシャー</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>21:00-21:30</t>
+          <t>21:30-22:00</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -1678,49 +1679,15 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>21:00-21:30</t>
+          <t>21:30-22:00</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Gさん</t>
+          <t>Fさん</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
-        <is>
-          <t>キャッシャー</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>21:30-22:00</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Eさん</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>バリスタ</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>21:30-22:00</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Gさん</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
         <is>
           <t>キャッシャー</t>
         </is>
@@ -1737,7 +1704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1791,19 +1758,19 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12:30-13:00</t>
+          <t>12:00-12:30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>バリスタ</t>
+          <t>フロア</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -1812,7 +1779,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13:00-13:30</t>
+          <t>12:30-13:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1833,7 +1800,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13:30-14:00</t>
+          <t>13:00-13:30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1849,6 +1816,189 @@
       </c>
       <c r="E5" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>13:00-13:30</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>13:30-14:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>15:00-15:30</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>15:30-16:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>名前</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>休憩開始</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>休憩終了</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cさん</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Dさん</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Eさん</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Fさん</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add pivot shift table
</commit_message>
<xml_diff>
--- a/split_30minute_result.xlsx
+++ b/split_30minute_result.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="シフト" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="欠員ログ" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="休憩予定" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="シフト表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="欠員ログ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="休憩予定" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1704,40 +1705,55 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>slot</t>
+          <t>時間</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>position</t>
+          <t>Aさん</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>required</t>
+          <t>Bさん</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>actual</t>
+          <t>Cさん</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>shortage</t>
+          <t>Dさん</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Eさん</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Fさん</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Gさん</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12:00-12:30</t>
+          <t>06:30-07:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1745,41 +1761,83 @@
           <t>バリスタ</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12:00-12:30</t>
+          <t>07:00-07:30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>フロア</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
-        <v>1</v>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12:30-13:00</t>
+          <t>07:30-08:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1787,20 +1845,41 @@
           <t>バリスタ</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13:00-13:30</t>
+          <t>08:00-08:30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1808,41 +1887,83 @@
           <t>バリスタ</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>1</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13:00-13:30</t>
+          <t>08:30-09:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>フロア</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1</v>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>13:30-14:00</t>
+          <t>09:00-09:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1850,56 +1971,1085 @@
           <t>バリスタ</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="n">
-        <v>1</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>15:00-15:30</t>
+          <t>09:30-10:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>キャッシャー</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>1</v>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>10:00-10:30</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>10:30-11:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>11:00-11:30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>11:30-12:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>12:00-12:30</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>12:30-13:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>13:00-13:30</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>13:30-14:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>14:00-14:30</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>14:30-15:00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>15:00-15:30</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>15:30-16:00</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>キャッシャー</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
-        <v>1</v>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>16:00-16:30</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>16:30-17:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>17:00-17:30</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>17:30-18:00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>18:00-18:30</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>18:30-19:00</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>19:00-19:30</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>19:30-20:00</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>20:00-20:30</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>20:30-21:00</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>21:00-21:30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>21:30-22:00</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>ー</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1913,6 +3063,215 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>actual</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>shortage</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12:00-12:30</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>12:00-12:30</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>12:30-13:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>13:00-13:30</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>13:00-13:30</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>フロア</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>13:30-14:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>バリスタ</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>15:00-15:30</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>15:30-16:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>キャッシャー</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>